<commit_message>
Trying to add updated wq data entry
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_point_wq.xlsx
+++ b/Data/tabular/YBLTE_point_wq.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Box\Yolo_Food_Web\Data\tabular\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kristinn\Downloads\wq\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2622D096-9AA3-4E21-AE39-D55F2AE30330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7082080F-BB4F-465A-96D5-4BA32ABAC219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="66">
   <si>
     <t>RowID</t>
   </si>
@@ -553,14 +553,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y130"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:Y144"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="10.54296875" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -637,7 +637,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -708,7 +708,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -776,7 +776,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -847,7 +847,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -916,7 +916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -985,7 +985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1539,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1677,7 +1677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2227,7 +2227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2780,7 +2780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2989,7 +2989,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3061,7 +3061,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3404,7 +3404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3614,7 +3614,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3683,7 +3683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3821,7 +3821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3957,7 +3957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4025,7 +4025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4094,7 +4094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4163,7 +4163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4304,7 +4304,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="55" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4442,7 +4442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4510,7 +4510,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4578,7 +4578,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4646,7 +4646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -4782,7 +4782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -4854,7 +4854,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -4926,7 +4926,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -4995,7 +4995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5067,7 +5067,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5139,7 +5139,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="67" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5208,7 +5208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5277,7 +5277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="70" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5417,7 +5417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5488,7 +5488,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="72" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -5556,7 +5556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -5627,7 +5627,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -5695,7 +5695,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -5764,7 +5764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -5833,7 +5833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -5905,7 +5905,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="78" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -5974,7 +5974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -6043,7 +6043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -6112,7 +6112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -6181,7 +6181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -6250,7 +6250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -6387,7 +6387,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="85" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -6456,7 +6456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -6528,7 +6528,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="87" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -6597,7 +6597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -6668,7 +6668,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="89" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -6737,7 +6737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -6799,14 +6799,14 @@
         <v>160074</v>
       </c>
       <c r="U90">
-        <f t="shared" ref="U90:U130" si="7">T90-S90</f>
+        <f t="shared" ref="U90:U143" si="7">T90-S90</f>
         <v>633</v>
       </c>
       <c r="V90">
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -6875,7 +6875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -6944,7 +6944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -7013,7 +7013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -7084,7 +7084,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="95" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -7153,7 +7153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -7222,7 +7222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -7290,7 +7290,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -7359,7 +7359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -7428,7 +7428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -7497,7 +7497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -7566,7 +7566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -7634,7 +7634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -7703,7 +7703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -7772,7 +7772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -7841,7 +7841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -7910,7 +7910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -7978,7 +7978,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -8047,7 +8047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -8116,7 +8116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -8185,7 +8185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -8254,7 +8254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -8323,7 +8323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -8395,7 +8395,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="114" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -8463,7 +8463,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="115" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -8535,7 +8535,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="116" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -8607,7 +8607,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="117" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -8676,7 +8676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -8745,7 +8745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -8814,7 +8814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -8883,7 +8883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -8952,7 +8952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -9024,7 +9024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -9093,7 +9093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -9162,7 +9162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -9234,7 +9234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -9306,7 +9306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -9377,7 +9377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -9448,7 +9448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -9520,7 +9520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -9586,6 +9586,968 @@
         <v>602</v>
       </c>
       <c r="V130">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>45</v>
+      </c>
+      <c r="C131" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D131" s="2">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="E131">
+        <v>9.85</v>
+      </c>
+      <c r="F131">
+        <v>91.3</v>
+      </c>
+      <c r="G131">
+        <v>10.32</v>
+      </c>
+      <c r="H131">
+        <v>736</v>
+      </c>
+      <c r="I131">
+        <v>478.584</v>
+      </c>
+      <c r="J131">
+        <v>0.36</v>
+      </c>
+      <c r="K131">
+        <v>8.2899999999999991</v>
+      </c>
+      <c r="L131">
+        <v>32.93</v>
+      </c>
+      <c r="M131">
+        <v>1.39</v>
+      </c>
+      <c r="N131">
+        <v>38.619999999999997</v>
+      </c>
+      <c r="O131">
+        <v>31.51</v>
+      </c>
+      <c r="P131">
+        <v>3.5</v>
+      </c>
+      <c r="Q131">
+        <v>30</v>
+      </c>
+      <c r="R131">
+        <v>4</v>
+      </c>
+      <c r="S131">
+        <v>12842</v>
+      </c>
+      <c r="T131">
+        <v>13501</v>
+      </c>
+      <c r="U131">
+        <f t="shared" si="7"/>
+        <v>659</v>
+      </c>
+      <c r="V131">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C132" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D132" s="2">
+        <v>0.39374999999999999</v>
+      </c>
+      <c r="E132">
+        <v>9.8130000000000006</v>
+      </c>
+      <c r="F132">
+        <v>92.4</v>
+      </c>
+      <c r="G132">
+        <v>10.48</v>
+      </c>
+      <c r="H132">
+        <v>167.9</v>
+      </c>
+      <c r="I132">
+        <v>109.167</v>
+      </c>
+      <c r="J132">
+        <v>0.08</v>
+      </c>
+      <c r="K132">
+        <v>7.89</v>
+      </c>
+      <c r="L132">
+        <v>12.86</v>
+      </c>
+      <c r="M132">
+        <v>0.21</v>
+      </c>
+      <c r="N132">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="O132">
+        <v>16.73</v>
+      </c>
+      <c r="P132">
+        <v>2</v>
+      </c>
+      <c r="Q132">
+        <v>30</v>
+      </c>
+      <c r="R132">
+        <v>4</v>
+      </c>
+      <c r="S132">
+        <v>13501</v>
+      </c>
+      <c r="T132">
+        <v>14135</v>
+      </c>
+      <c r="U132">
+        <f t="shared" si="7"/>
+        <v>634</v>
+      </c>
+      <c r="V132">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>29</v>
+      </c>
+      <c r="C133" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D133" s="2">
+        <v>0.40625</v>
+      </c>
+      <c r="E133">
+        <v>10.066000000000001</v>
+      </c>
+      <c r="F133">
+        <v>94</v>
+      </c>
+      <c r="G133">
+        <v>10.58</v>
+      </c>
+      <c r="H133">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="I133">
+        <v>209.36799999999999</v>
+      </c>
+      <c r="J133">
+        <v>0.15</v>
+      </c>
+      <c r="K133">
+        <v>7.8</v>
+      </c>
+      <c r="L133">
+        <v>9.26</v>
+      </c>
+      <c r="M133">
+        <v>0.67</v>
+      </c>
+      <c r="N133">
+        <v>10.46</v>
+      </c>
+      <c r="O133">
+        <v>33.049999999999997</v>
+      </c>
+      <c r="P133">
+        <v>1.5</v>
+      </c>
+      <c r="Q133">
+        <v>30</v>
+      </c>
+      <c r="R133">
+        <v>4</v>
+      </c>
+      <c r="S133">
+        <v>14135</v>
+      </c>
+      <c r="T133">
+        <v>14793</v>
+      </c>
+      <c r="U133">
+        <f t="shared" si="7"/>
+        <v>658</v>
+      </c>
+      <c r="V133">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>30</v>
+      </c>
+      <c r="C134" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D134" s="2">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="E134">
+        <v>9.9670000000000005</v>
+      </c>
+      <c r="F134">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="G134">
+        <v>7.82</v>
+      </c>
+      <c r="H134">
+        <v>596</v>
+      </c>
+      <c r="I134">
+        <v>387.47800000000001</v>
+      </c>
+      <c r="J134">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="K134">
+        <v>7.81</v>
+      </c>
+      <c r="L134">
+        <v>25.61</v>
+      </c>
+      <c r="M134">
+        <v>0.59</v>
+      </c>
+      <c r="N134">
+        <v>7.37</v>
+      </c>
+      <c r="O134">
+        <v>76.28</v>
+      </c>
+      <c r="P134">
+        <v>4.5</v>
+      </c>
+      <c r="Q134">
+        <v>30</v>
+      </c>
+      <c r="R134">
+        <v>4</v>
+      </c>
+      <c r="S134">
+        <v>14793</v>
+      </c>
+      <c r="T134">
+        <v>15583</v>
+      </c>
+      <c r="U134">
+        <f t="shared" si="7"/>
+        <v>790</v>
+      </c>
+      <c r="V134">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>44</v>
+      </c>
+      <c r="C135" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D135" s="2">
+        <v>0.45555555555555555</v>
+      </c>
+      <c r="E135">
+        <v>10.141999999999999</v>
+      </c>
+      <c r="F135">
+        <v>108.1</v>
+      </c>
+      <c r="G135">
+        <v>12.15</v>
+      </c>
+      <c r="H135">
+        <v>552</v>
+      </c>
+      <c r="I135">
+        <v>358.88799999999998</v>
+      </c>
+      <c r="J135">
+        <v>0.27</v>
+      </c>
+      <c r="K135">
+        <v>8.4600000000000009</v>
+      </c>
+      <c r="L135">
+        <v>14.85</v>
+      </c>
+      <c r="M135">
+        <v>0.73</v>
+      </c>
+      <c r="N135">
+        <v>11.81</v>
+      </c>
+      <c r="O135">
+        <v>71.61</v>
+      </c>
+      <c r="P135">
+        <v>3.5</v>
+      </c>
+      <c r="Q135">
+        <v>30</v>
+      </c>
+      <c r="R135">
+        <v>4</v>
+      </c>
+      <c r="S135">
+        <v>15595</v>
+      </c>
+      <c r="T135">
+        <v>16275</v>
+      </c>
+      <c r="U135">
+        <f t="shared" si="7"/>
+        <v>680</v>
+      </c>
+      <c r="V135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>56</v>
+      </c>
+      <c r="C136" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D136" s="2">
+        <v>0.47430555555555554</v>
+      </c>
+      <c r="E136">
+        <v>10.645</v>
+      </c>
+      <c r="F136">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="G136">
+        <v>8.66</v>
+      </c>
+      <c r="H136">
+        <v>203</v>
+      </c>
+      <c r="I136">
+        <v>132.268</v>
+      </c>
+      <c r="J136">
+        <v>0.1</v>
+      </c>
+      <c r="K136">
+        <v>7.65</v>
+      </c>
+      <c r="L136">
+        <v>12.03</v>
+      </c>
+      <c r="M136">
+        <v>0.39</v>
+      </c>
+      <c r="N136">
+        <v>4.46</v>
+      </c>
+      <c r="O136">
+        <v>35.06</v>
+      </c>
+      <c r="P136">
+        <v>5</v>
+      </c>
+      <c r="Q136">
+        <v>30</v>
+      </c>
+      <c r="R136">
+        <v>4</v>
+      </c>
+      <c r="S136">
+        <v>16279</v>
+      </c>
+      <c r="T136">
+        <v>16929</v>
+      </c>
+      <c r="U136">
+        <f t="shared" si="7"/>
+        <v>650</v>
+      </c>
+      <c r="V136">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>31</v>
+      </c>
+      <c r="C137" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D137" s="2">
+        <v>0.5083333333333333</v>
+      </c>
+      <c r="E137">
+        <v>10.531000000000001</v>
+      </c>
+      <c r="F137">
+        <v>79</v>
+      </c>
+      <c r="G137">
+        <v>8.7899999999999991</v>
+      </c>
+      <c r="H137">
+        <v>547</v>
+      </c>
+      <c r="I137">
+        <v>355.83100000000002</v>
+      </c>
+      <c r="J137">
+        <v>0.27</v>
+      </c>
+      <c r="K137">
+        <v>7.89</v>
+      </c>
+      <c r="L137">
+        <v>22.32</v>
+      </c>
+      <c r="M137">
+        <v>0.72</v>
+      </c>
+      <c r="N137">
+        <v>13.97</v>
+      </c>
+      <c r="O137">
+        <v>70.540000000000006</v>
+      </c>
+      <c r="P137">
+        <v>4</v>
+      </c>
+      <c r="Q137">
+        <v>30</v>
+      </c>
+      <c r="R137">
+        <v>4</v>
+      </c>
+      <c r="S137">
+        <v>17527</v>
+      </c>
+      <c r="T137">
+        <v>18105</v>
+      </c>
+      <c r="U137">
+        <f t="shared" si="7"/>
+        <v>578</v>
+      </c>
+      <c r="V137">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>32</v>
+      </c>
+      <c r="C138" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D138" s="2">
+        <v>0.52986111111111112</v>
+      </c>
+      <c r="E138">
+        <v>10.215999999999999</v>
+      </c>
+      <c r="F138">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="G138">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="H138">
+        <v>529</v>
+      </c>
+      <c r="I138">
+        <v>344.15</v>
+      </c>
+      <c r="J138">
+        <v>0.26</v>
+      </c>
+      <c r="K138">
+        <v>7.89</v>
+      </c>
+      <c r="L138">
+        <v>21.45</v>
+      </c>
+      <c r="M138">
+        <v>0.73</v>
+      </c>
+      <c r="N138">
+        <v>15.08</v>
+      </c>
+      <c r="O138">
+        <v>71.5</v>
+      </c>
+      <c r="P138">
+        <v>4.5</v>
+      </c>
+      <c r="Q138">
+        <v>30</v>
+      </c>
+      <c r="R138">
+        <v>4</v>
+      </c>
+      <c r="S138">
+        <v>18105</v>
+      </c>
+      <c r="T138">
+        <v>18830</v>
+      </c>
+      <c r="U138">
+        <f t="shared" si="7"/>
+        <v>725</v>
+      </c>
+      <c r="V138">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>33</v>
+      </c>
+      <c r="C139" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D139" s="2">
+        <v>0.55833333333333335</v>
+      </c>
+      <c r="E139">
+        <v>10.455</v>
+      </c>
+      <c r="F139">
+        <v>78.7</v>
+      </c>
+      <c r="G139">
+        <v>8.77</v>
+      </c>
+      <c r="H139">
+        <v>519</v>
+      </c>
+      <c r="I139">
+        <v>337.15699999999998</v>
+      </c>
+      <c r="J139">
+        <v>0.25</v>
+      </c>
+      <c r="K139">
+        <v>7.85</v>
+      </c>
+      <c r="L139">
+        <v>21.25</v>
+      </c>
+      <c r="M139">
+        <v>0.7</v>
+      </c>
+      <c r="N139">
+        <v>13.62</v>
+      </c>
+      <c r="O139">
+        <v>73.94</v>
+      </c>
+      <c r="P139">
+        <v>4.5</v>
+      </c>
+      <c r="Q139">
+        <v>30</v>
+      </c>
+      <c r="R139">
+        <v>4</v>
+      </c>
+      <c r="S139">
+        <v>18888</v>
+      </c>
+      <c r="T139">
+        <v>19502</v>
+      </c>
+      <c r="U139">
+        <f t="shared" si="7"/>
+        <v>614</v>
+      </c>
+      <c r="V139">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>41</v>
+      </c>
+      <c r="C140" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D140" s="2">
+        <v>0.39444444444444443</v>
+      </c>
+      <c r="E140">
+        <v>7.9669999999999996</v>
+      </c>
+      <c r="F140">
+        <v>65.3</v>
+      </c>
+      <c r="G140">
+        <v>7.73</v>
+      </c>
+      <c r="H140">
+        <v>501</v>
+      </c>
+      <c r="I140">
+        <v>325.86</v>
+      </c>
+      <c r="J140">
+        <v>0.24</v>
+      </c>
+      <c r="K140">
+        <v>7.63</v>
+      </c>
+      <c r="L140">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="M140">
+        <v>0.19</v>
+      </c>
+      <c r="N140">
+        <v>2.09</v>
+      </c>
+      <c r="O140">
+        <v>77.02</v>
+      </c>
+      <c r="P140">
+        <v>5</v>
+      </c>
+      <c r="Q140">
+        <v>15</v>
+      </c>
+      <c r="R140">
+        <v>4</v>
+      </c>
+      <c r="S140" t="s">
+        <v>24</v>
+      </c>
+      <c r="T140" t="s">
+        <v>24</v>
+      </c>
+      <c r="U140" t="s">
+        <v>24</v>
+      </c>
+      <c r="V140">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>42</v>
+      </c>
+      <c r="C141" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D141" s="2">
+        <v>0.41249999999999998</v>
+      </c>
+      <c r="E141">
+        <v>9.9480000000000004</v>
+      </c>
+      <c r="F141">
+        <v>62.1</v>
+      </c>
+      <c r="G141">
+        <v>7</v>
+      </c>
+      <c r="H141">
+        <v>586</v>
+      </c>
+      <c r="I141">
+        <v>380.60300000000001</v>
+      </c>
+      <c r="J141">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="K141">
+        <v>7.68</v>
+      </c>
+      <c r="L141">
+        <v>20.83</v>
+      </c>
+      <c r="M141">
+        <v>0.44</v>
+      </c>
+      <c r="N141">
+        <v>7.1</v>
+      </c>
+      <c r="O141">
+        <v>78.3</v>
+      </c>
+      <c r="P141" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q141" t="s">
+        <v>24</v>
+      </c>
+      <c r="R141" t="s">
+        <v>24</v>
+      </c>
+      <c r="S141" t="s">
+        <v>24</v>
+      </c>
+      <c r="T141" t="s">
+        <v>24</v>
+      </c>
+      <c r="U141" t="s">
+        <v>24</v>
+      </c>
+      <c r="V141" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="142" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>61</v>
+      </c>
+      <c r="C142" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D142" s="2">
+        <v>0.44027777777777777</v>
+      </c>
+      <c r="E142">
+        <v>9.0920000000000005</v>
+      </c>
+      <c r="F142">
+        <v>96.4</v>
+      </c>
+      <c r="G142">
+        <v>11.11</v>
+      </c>
+      <c r="H142">
+        <v>304.89999999999998</v>
+      </c>
+      <c r="I142">
+        <v>198.154</v>
+      </c>
+      <c r="J142">
+        <v>0.15</v>
+      </c>
+      <c r="K142">
+        <v>7.82</v>
+      </c>
+      <c r="L142">
+        <v>57.66</v>
+      </c>
+      <c r="M142">
+        <v>0.6</v>
+      </c>
+      <c r="N142">
+        <v>15.26</v>
+      </c>
+      <c r="O142">
+        <v>41.66</v>
+      </c>
+      <c r="P142">
+        <v>4</v>
+      </c>
+      <c r="Q142">
+        <v>15</v>
+      </c>
+      <c r="R142" t="s">
+        <v>24</v>
+      </c>
+      <c r="S142" t="s">
+        <v>24</v>
+      </c>
+      <c r="T142" t="s">
+        <v>24</v>
+      </c>
+      <c r="U142" t="s">
+        <v>24</v>
+      </c>
+      <c r="V142">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>34</v>
+      </c>
+      <c r="C143" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D143" s="2">
+        <v>0.51875000000000004</v>
+      </c>
+      <c r="E143">
+        <v>11.422000000000001</v>
+      </c>
+      <c r="F143">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="G143">
+        <v>7.35</v>
+      </c>
+      <c r="H143">
+        <v>417.2</v>
+      </c>
+      <c r="I143">
+        <v>271.19799999999998</v>
+      </c>
+      <c r="J143">
+        <v>0.2</v>
+      </c>
+      <c r="K143">
+        <v>7.42</v>
+      </c>
+      <c r="L143">
+        <v>4.58</v>
+      </c>
+      <c r="M143">
+        <v>0.25</v>
+      </c>
+      <c r="N143">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="O143">
+        <v>88.42</v>
+      </c>
+      <c r="P143">
+        <v>5</v>
+      </c>
+      <c r="Q143">
+        <v>30</v>
+      </c>
+      <c r="R143">
+        <v>4</v>
+      </c>
+      <c r="S143">
+        <v>8835</v>
+      </c>
+      <c r="T143">
+        <v>9472</v>
+      </c>
+      <c r="U143">
+        <f t="shared" si="7"/>
+        <v>637</v>
+      </c>
+      <c r="V143">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>36</v>
+      </c>
+      <c r="C144" s="1">
+        <v>46049</v>
+      </c>
+      <c r="D144" s="2">
+        <v>0.56666666666666665</v>
+      </c>
+      <c r="E144">
+        <v>14.577999999999999</v>
+      </c>
+      <c r="F144">
+        <v>54.8</v>
+      </c>
+      <c r="G144">
+        <v>5.58</v>
+      </c>
+      <c r="H144">
+        <v>359.4</v>
+      </c>
+      <c r="I144">
+        <v>233.63200000000001</v>
+      </c>
+      <c r="J144">
+        <v>0.17</v>
+      </c>
+      <c r="K144">
+        <v>7.25</v>
+      </c>
+      <c r="L144">
+        <v>20.260000000000002</v>
+      </c>
+      <c r="M144">
+        <v>0.11</v>
+      </c>
+      <c r="N144">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="O144">
+        <v>58.41</v>
+      </c>
+      <c r="P144">
+        <v>5</v>
+      </c>
+      <c r="Q144">
+        <v>15</v>
+      </c>
+      <c r="R144">
+        <v>4</v>
+      </c>
+      <c r="S144" t="s">
+        <v>24</v>
+      </c>
+      <c r="T144" t="s">
+        <v>24</v>
+      </c>
+      <c r="U144" t="s">
+        <v>24</v>
+      </c>
+      <c r="V144">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updating YBLTE wq data
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_point_wq.xlsx
+++ b/Data/tabular/YBLTE_point_wq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kristinn\Downloads\wq\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kristinn\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7082080F-BB4F-465A-96D5-4BA32ABAC219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{DF4F414E-7754-416B-A942-8B6CCBBB419D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="67">
   <si>
     <t>RowID</t>
   </si>
@@ -235,15 +235,24 @@
   <si>
     <t>Flow meter rotations suspect</t>
   </si>
+  <si>
+    <t>Missing cod end on net</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -553,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y144"/>
+  <dimension ref="A1:Y158"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -6799,7 +6808,7 @@
         <v>160074</v>
       </c>
       <c r="U90">
-        <f t="shared" ref="U90:U143" si="7">T90-S90</f>
+        <f t="shared" ref="U90:U153" si="7">T90-S90</f>
         <v>633</v>
       </c>
       <c r="V90">
@@ -10398,8 +10407,8 @@
       <c r="Q142">
         <v>15</v>
       </c>
-      <c r="R142" t="s">
-        <v>24</v>
+      <c r="R142">
+        <v>4</v>
       </c>
       <c r="S142" t="s">
         <v>24</v>
@@ -10551,7 +10560,973 @@
         <v>1</v>
       </c>
     </row>
+    <row r="145" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>45</v>
+      </c>
+      <c r="C145" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D145" s="2">
+        <v>0.34513888888888888</v>
+      </c>
+      <c r="E145">
+        <v>11.208</v>
+      </c>
+      <c r="F145">
+        <v>90.5</v>
+      </c>
+      <c r="G145">
+        <v>9.9</v>
+      </c>
+      <c r="H145">
+        <v>873</v>
+      </c>
+      <c r="I145">
+        <v>567.64200000000005</v>
+      </c>
+      <c r="J145">
+        <v>0.43</v>
+      </c>
+      <c r="K145">
+        <v>8.27</v>
+      </c>
+      <c r="L145">
+        <v>16.25</v>
+      </c>
+      <c r="M145">
+        <v>0.38</v>
+      </c>
+      <c r="N145">
+        <v>14.2</v>
+      </c>
+      <c r="O145">
+        <v>24.33</v>
+      </c>
+      <c r="P145">
+        <v>3.5</v>
+      </c>
+      <c r="Q145">
+        <v>30</v>
+      </c>
+      <c r="R145">
+        <v>4</v>
+      </c>
+      <c r="S145">
+        <v>175305</v>
+      </c>
+      <c r="T145">
+        <v>175968</v>
+      </c>
+      <c r="U145">
+        <f t="shared" si="7"/>
+        <v>663</v>
+      </c>
+      <c r="V145">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>27</v>
+      </c>
+      <c r="C146" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D146" s="2">
+        <v>0.37430555555555556</v>
+      </c>
+      <c r="E146">
+        <v>10.978999999999999</v>
+      </c>
+      <c r="F146">
+        <v>98.1</v>
+      </c>
+      <c r="G146">
+        <v>10.82</v>
+      </c>
+      <c r="H146">
+        <v>170.3</v>
+      </c>
+      <c r="I146">
+        <v>110.70699999999999</v>
+      </c>
+      <c r="J146">
+        <v>0.08</v>
+      </c>
+      <c r="K146">
+        <v>7.83</v>
+      </c>
+      <c r="L146">
+        <v>11.62</v>
+      </c>
+      <c r="M146">
+        <v>0.2</v>
+      </c>
+      <c r="N146">
+        <v>2.13</v>
+      </c>
+      <c r="O146">
+        <v>13.9</v>
+      </c>
+      <c r="P146">
+        <v>2</v>
+      </c>
+      <c r="Q146">
+        <v>30</v>
+      </c>
+      <c r="R146">
+        <v>4</v>
+      </c>
+      <c r="S146">
+        <v>175968</v>
+      </c>
+      <c r="T146">
+        <v>176612</v>
+      </c>
+      <c r="U146">
+        <f t="shared" si="7"/>
+        <v>644</v>
+      </c>
+      <c r="V146">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>29</v>
+      </c>
+      <c r="C147" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D147" s="2">
+        <v>0.39513888888888887</v>
+      </c>
+      <c r="E147">
+        <v>10.8</v>
+      </c>
+      <c r="F147">
+        <v>94.7</v>
+      </c>
+      <c r="G147">
+        <v>10.49</v>
+      </c>
+      <c r="H147">
+        <v>170</v>
+      </c>
+      <c r="I147">
+        <v>110.511</v>
+      </c>
+      <c r="J147">
+        <v>0.08</v>
+      </c>
+      <c r="K147">
+        <v>7.7</v>
+      </c>
+      <c r="L147">
+        <v>11.47</v>
+      </c>
+      <c r="M147">
+        <v>0.11</v>
+      </c>
+      <c r="N147">
+        <v>2.04</v>
+      </c>
+      <c r="O147">
+        <v>14.12</v>
+      </c>
+      <c r="P147">
+        <v>1.5</v>
+      </c>
+      <c r="Q147">
+        <v>30</v>
+      </c>
+      <c r="R147">
+        <v>4</v>
+      </c>
+      <c r="S147">
+        <v>176612</v>
+      </c>
+      <c r="T147">
+        <v>177218</v>
+      </c>
+      <c r="U147">
+        <f t="shared" si="7"/>
+        <v>606</v>
+      </c>
+      <c r="V147">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>30</v>
+      </c>
+      <c r="C148" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D148" s="2">
+        <v>0.41944444444444445</v>
+      </c>
+      <c r="E148">
+        <v>11.53</v>
+      </c>
+      <c r="F148">
+        <v>77.7</v>
+      </c>
+      <c r="G148">
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="H148">
+        <v>565</v>
+      </c>
+      <c r="I148">
+        <v>367.40300000000002</v>
+      </c>
+      <c r="J148">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="K148">
+        <v>7.82</v>
+      </c>
+      <c r="L148">
+        <v>23.18</v>
+      </c>
+      <c r="M148">
+        <v>0.3</v>
+      </c>
+      <c r="N148">
+        <v>5.79</v>
+      </c>
+      <c r="O148">
+        <v>61.2</v>
+      </c>
+      <c r="P148">
+        <v>3</v>
+      </c>
+      <c r="Q148">
+        <v>30</v>
+      </c>
+      <c r="R148">
+        <v>4</v>
+      </c>
+      <c r="S148">
+        <v>177218</v>
+      </c>
+      <c r="T148">
+        <v>177785</v>
+      </c>
+      <c r="U148">
+        <f t="shared" si="7"/>
+        <v>567</v>
+      </c>
+      <c r="V148">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>44</v>
+      </c>
+      <c r="C149" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D149" s="2">
+        <v>0.44513888888888886</v>
+      </c>
+      <c r="E149">
+        <v>12.92</v>
+      </c>
+      <c r="F149">
+        <v>114.7</v>
+      </c>
+      <c r="G149">
+        <v>12.09</v>
+      </c>
+      <c r="H149">
+        <v>620</v>
+      </c>
+      <c r="I149">
+        <v>402.85700000000003</v>
+      </c>
+      <c r="J149">
+        <v>0.3</v>
+      </c>
+      <c r="K149">
+        <v>8.67</v>
+      </c>
+      <c r="L149">
+        <v>10.67</v>
+      </c>
+      <c r="M149">
+        <v>0.35</v>
+      </c>
+      <c r="N149">
+        <v>9.11</v>
+      </c>
+      <c r="O149">
+        <v>62.49</v>
+      </c>
+      <c r="P149">
+        <v>5</v>
+      </c>
+      <c r="Q149">
+        <v>30</v>
+      </c>
+      <c r="R149">
+        <v>4</v>
+      </c>
+      <c r="S149">
+        <v>177785</v>
+      </c>
+      <c r="T149">
+        <v>178424</v>
+      </c>
+      <c r="U149">
+        <f t="shared" si="7"/>
+        <v>639</v>
+      </c>
+      <c r="V149">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>56</v>
+      </c>
+      <c r="C150" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D150" s="2">
+        <v>0.46736111111111112</v>
+      </c>
+      <c r="E150">
+        <v>13.569000000000001</v>
+      </c>
+      <c r="F150">
+        <v>90</v>
+      </c>
+      <c r="G150">
+        <v>9.35</v>
+      </c>
+      <c r="H150">
+        <v>504</v>
+      </c>
+      <c r="I150">
+        <v>327.57299999999998</v>
+      </c>
+      <c r="J150">
+        <v>0.24</v>
+      </c>
+      <c r="K150">
+        <v>8.1</v>
+      </c>
+      <c r="L150">
+        <v>78.16</v>
+      </c>
+      <c r="M150">
+        <v>1.29</v>
+      </c>
+      <c r="N150">
+        <v>25.99</v>
+      </c>
+      <c r="O150">
+        <v>30.71</v>
+      </c>
+      <c r="P150">
+        <v>5</v>
+      </c>
+      <c r="Q150">
+        <v>30</v>
+      </c>
+      <c r="R150">
+        <v>4</v>
+      </c>
+      <c r="S150">
+        <v>178424</v>
+      </c>
+      <c r="T150">
+        <v>179033</v>
+      </c>
+      <c r="U150">
+        <f t="shared" si="7"/>
+        <v>609</v>
+      </c>
+      <c r="V150">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>31</v>
+      </c>
+      <c r="C151" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D151" s="2">
+        <v>0.5083333333333333</v>
+      </c>
+      <c r="E151">
+        <v>12.526</v>
+      </c>
+      <c r="F151">
+        <v>77</v>
+      </c>
+      <c r="G151">
+        <v>8.18</v>
+      </c>
+      <c r="H151">
+        <v>567</v>
+      </c>
+      <c r="I151">
+        <v>368.50900000000001</v>
+      </c>
+      <c r="J151">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="K151">
+        <v>7.84</v>
+      </c>
+      <c r="L151">
+        <v>22.64</v>
+      </c>
+      <c r="M151">
+        <v>0.3</v>
+      </c>
+      <c r="N151">
+        <v>7.58</v>
+      </c>
+      <c r="O151">
+        <v>58.77</v>
+      </c>
+      <c r="P151">
+        <v>3.5</v>
+      </c>
+      <c r="Q151">
+        <v>30</v>
+      </c>
+      <c r="R151">
+        <v>4</v>
+      </c>
+      <c r="S151">
+        <v>179033</v>
+      </c>
+      <c r="T151">
+        <v>179659</v>
+      </c>
+      <c r="U151">
+        <f t="shared" si="7"/>
+        <v>626</v>
+      </c>
+      <c r="V151">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>32</v>
+      </c>
+      <c r="C152" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D152" s="2">
+        <v>0.52430555555555558</v>
+      </c>
+      <c r="E152">
+        <v>12.545999999999999</v>
+      </c>
+      <c r="F152">
+        <v>81.099999999999994</v>
+      </c>
+      <c r="G152">
+        <v>8.6199999999999992</v>
+      </c>
+      <c r="H152">
+        <v>578</v>
+      </c>
+      <c r="I152">
+        <v>375.541</v>
+      </c>
+      <c r="J152">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="K152">
+        <v>7.82</v>
+      </c>
+      <c r="L152">
+        <v>22.1</v>
+      </c>
+      <c r="M152">
+        <v>0.35</v>
+      </c>
+      <c r="N152">
+        <v>9.1</v>
+      </c>
+      <c r="O152">
+        <v>60.21</v>
+      </c>
+      <c r="P152">
+        <v>3.5</v>
+      </c>
+      <c r="Q152">
+        <v>30</v>
+      </c>
+      <c r="R152">
+        <v>4</v>
+      </c>
+      <c r="S152">
+        <v>179659</v>
+      </c>
+      <c r="T152">
+        <v>180265</v>
+      </c>
+      <c r="U152">
+        <f t="shared" si="7"/>
+        <v>606</v>
+      </c>
+      <c r="V152">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>33</v>
+      </c>
+      <c r="C153" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D153" s="2">
+        <v>0.5493055555555556</v>
+      </c>
+      <c r="E153">
+        <v>12.407999999999999</v>
+      </c>
+      <c r="F153">
+        <v>77</v>
+      </c>
+      <c r="G153">
+        <v>8.2100000000000009</v>
+      </c>
+      <c r="H153">
+        <v>575</v>
+      </c>
+      <c r="I153">
+        <v>373.70499999999998</v>
+      </c>
+      <c r="J153">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="K153">
+        <v>7.8</v>
+      </c>
+      <c r="L153">
+        <v>18.16</v>
+      </c>
+      <c r="M153">
+        <v>0.4</v>
+      </c>
+      <c r="N153">
+        <v>8.65</v>
+      </c>
+      <c r="O153">
+        <v>58.95</v>
+      </c>
+      <c r="P153">
+        <v>4</v>
+      </c>
+      <c r="Q153">
+        <v>30</v>
+      </c>
+      <c r="R153">
+        <v>4</v>
+      </c>
+      <c r="S153">
+        <v>180265</v>
+      </c>
+      <c r="T153">
+        <v>180858</v>
+      </c>
+      <c r="U153">
+        <f t="shared" si="7"/>
+        <v>593</v>
+      </c>
+      <c r="V153">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="s">
+        <v>41</v>
+      </c>
+      <c r="C154" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D154" s="2">
+        <v>0.36527777777777776</v>
+      </c>
+      <c r="E154">
+        <v>11.74</v>
+      </c>
+      <c r="F154">
+        <v>44</v>
+      </c>
+      <c r="G154">
+        <v>4.76</v>
+      </c>
+      <c r="H154">
+        <v>537</v>
+      </c>
+      <c r="I154">
+        <v>348.80399999999997</v>
+      </c>
+      <c r="J154">
+        <v>0.26</v>
+      </c>
+      <c r="K154">
+        <v>7.47</v>
+      </c>
+      <c r="L154">
+        <v>5.03</v>
+      </c>
+      <c r="M154">
+        <v>0.2</v>
+      </c>
+      <c r="N154">
+        <v>1.73</v>
+      </c>
+      <c r="O154">
+        <v>82.7</v>
+      </c>
+      <c r="P154" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q154" t="s">
+        <v>24</v>
+      </c>
+      <c r="R154" t="s">
+        <v>24</v>
+      </c>
+      <c r="S154" t="s">
+        <v>24</v>
+      </c>
+      <c r="T154" t="s">
+        <v>24</v>
+      </c>
+      <c r="U154" t="s">
+        <v>24</v>
+      </c>
+      <c r="V154">
+        <v>1</v>
+      </c>
+      <c r="Y154" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="155" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="s">
+        <v>41</v>
+      </c>
+      <c r="C155" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D155" s="2">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="E155">
+        <v>12.023</v>
+      </c>
+      <c r="F155">
+        <v>46.1</v>
+      </c>
+      <c r="G155">
+        <v>4.96</v>
+      </c>
+      <c r="H155">
+        <v>539</v>
+      </c>
+      <c r="I155">
+        <v>350.10599999999999</v>
+      </c>
+      <c r="J155">
+        <v>0.26</v>
+      </c>
+      <c r="K155">
+        <v>7.5</v>
+      </c>
+      <c r="L155">
+        <v>7.44</v>
+      </c>
+      <c r="M155">
+        <v>0.16</v>
+      </c>
+      <c r="N155">
+        <v>1.84</v>
+      </c>
+      <c r="O155">
+        <v>81.06</v>
+      </c>
+      <c r="P155">
+        <v>4.5</v>
+      </c>
+      <c r="Q155">
+        <v>30</v>
+      </c>
+      <c r="R155">
+        <v>4</v>
+      </c>
+      <c r="S155">
+        <v>9955</v>
+      </c>
+      <c r="T155">
+        <v>10535</v>
+      </c>
+      <c r="U155">
+        <f t="shared" ref="U154:U158" si="8">T155-S155</f>
+        <v>580</v>
+      </c>
+      <c r="V155">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="s">
+        <v>42</v>
+      </c>
+      <c r="C156" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D156" s="2">
+        <v>0.44583333333333336</v>
+      </c>
+      <c r="E156">
+        <v>12.367000000000001</v>
+      </c>
+      <c r="F156">
+        <v>81.7</v>
+      </c>
+      <c r="G156">
+        <v>8.7200000000000006</v>
+      </c>
+      <c r="H156">
+        <v>648</v>
+      </c>
+      <c r="I156">
+        <v>421.36500000000001</v>
+      </c>
+      <c r="J156">
+        <v>0.32</v>
+      </c>
+      <c r="K156">
+        <v>7.93</v>
+      </c>
+      <c r="L156">
+        <v>20.39</v>
+      </c>
+      <c r="M156">
+        <v>0.38</v>
+      </c>
+      <c r="N156">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="O156">
+        <v>81.96</v>
+      </c>
+      <c r="P156" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q156" t="s">
+        <v>24</v>
+      </c>
+      <c r="R156" t="s">
+        <v>24</v>
+      </c>
+      <c r="S156" t="s">
+        <v>24</v>
+      </c>
+      <c r="T156" t="s">
+        <v>24</v>
+      </c>
+      <c r="U156" t="s">
+        <v>24</v>
+      </c>
+      <c r="V156" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="157" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="s">
+        <v>61</v>
+      </c>
+      <c r="C157" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D157" s="2">
+        <v>0.48888888888888887</v>
+      </c>
+      <c r="E157">
+        <v>12.903</v>
+      </c>
+      <c r="F157">
+        <v>98.1</v>
+      </c>
+      <c r="G157">
+        <v>10.35</v>
+      </c>
+      <c r="H157">
+        <v>374.2</v>
+      </c>
+      <c r="I157">
+        <v>243.21199999999999</v>
+      </c>
+      <c r="J157">
+        <v>0.18</v>
+      </c>
+      <c r="K157">
+        <v>7.73</v>
+      </c>
+      <c r="L157">
+        <v>78.28</v>
+      </c>
+      <c r="M157">
+        <v>0.99</v>
+      </c>
+      <c r="N157">
+        <v>17.239999999999998</v>
+      </c>
+      <c r="O157">
+        <v>45.8</v>
+      </c>
+      <c r="P157">
+        <v>4.5</v>
+      </c>
+      <c r="Q157">
+        <v>15</v>
+      </c>
+      <c r="R157">
+        <v>4</v>
+      </c>
+      <c r="S157" t="s">
+        <v>24</v>
+      </c>
+      <c r="T157" t="s">
+        <v>24</v>
+      </c>
+      <c r="U157" t="s">
+        <v>24</v>
+      </c>
+      <c r="V157">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="s">
+        <v>34</v>
+      </c>
+      <c r="C158" s="1">
+        <v>46056</v>
+      </c>
+      <c r="D158" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="E158">
+        <v>14.545</v>
+      </c>
+      <c r="F158">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="G158">
+        <v>7.79</v>
+      </c>
+      <c r="H158">
+        <v>549</v>
+      </c>
+      <c r="I158">
+        <v>357.14499999999998</v>
+      </c>
+      <c r="J158">
+        <v>0.27</v>
+      </c>
+      <c r="K158">
+        <v>7.43</v>
+      </c>
+      <c r="L158">
+        <v>5.17</v>
+      </c>
+      <c r="M158">
+        <v>0.22</v>
+      </c>
+      <c r="N158">
+        <v>2.9</v>
+      </c>
+      <c r="O158">
+        <v>89.15</v>
+      </c>
+      <c r="P158">
+        <v>5</v>
+      </c>
+      <c r="Q158">
+        <v>15</v>
+      </c>
+      <c r="R158">
+        <v>4</v>
+      </c>
+      <c r="S158" t="s">
+        <v>24</v>
+      </c>
+      <c r="T158" t="s">
+        <v>24</v>
+      </c>
+      <c r="U158" t="s">
+        <v>24</v>
+      </c>
+      <c r="V158">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
updating sites and point wq excels in github
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_point_wq.xlsx
+++ b/Data/tabular/YBLTE_point_wq.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Box\Yolo_Food_Web\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="485" documentId="13_ncr:1_{3AFD425C-1797-475E-8EFF-D332B24BA87F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE017823-1393-460C-872D-4976FEACD737}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2416E154-FDFB-4B9B-878A-86C1F8869F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -267,7 +267,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -600,13 +600,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z210"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="24" max="25" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
+    <col min="24" max="25" width="10.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -686,7 +686,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -760,7 +760,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -831,7 +831,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -905,7 +905,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -977,7 +977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1411,7 +1411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:26">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:26">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:26">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:26">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2058,7 +2058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:26">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:26">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:26">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:26">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:26">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:26">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:26">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:26">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:26">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:26">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2779,7 +2779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:26">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2851,7 +2851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:26">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:26">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:26">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:26">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3140,7 +3140,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:26">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="1:26">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:26">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3359,7 +3359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:26">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:26">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3501,7 +3501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:26">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:26">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:26">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3717,7 +3717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:26">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3792,7 +3792,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:26">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3864,7 +3864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:26">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:26">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4008,7 +4008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:26">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4079,7 +4079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:26">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:26">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4221,7 +4221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:26">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4293,7 +4293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:26">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4365,7 +4365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:26">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:26">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:26">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4584,7 +4584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:26">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4656,7 +4656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:26">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4727,7 +4727,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:26">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4798,7 +4798,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="59" spans="1:26">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4869,7 +4869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:26">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4940,7 +4940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:26">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:26">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5086,7 +5086,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:26">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5161,7 +5161,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:26">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:26">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5308,7 +5308,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="66" spans="1:26">
+    <row r="66" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5383,7 +5383,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:26">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5455,7 +5455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:26">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5527,7 +5527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:26">
+    <row r="69" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="70" spans="1:26">
+    <row r="70" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5673,7 +5673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:26">
+    <row r="71" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5747,7 +5747,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="72" spans="1:26">
+    <row r="72" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -5818,7 +5818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:26">
+    <row r="73" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -5892,7 +5892,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="74" spans="1:26">
+    <row r="74" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -5963,7 +5963,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="75" spans="1:26">
+    <row r="75" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -6035,7 +6035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:26">
+    <row r="76" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -6107,7 +6107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:26">
+    <row r="77" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -6182,7 +6182,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:26">
+    <row r="78" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -6254,7 +6254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:26">
+    <row r="79" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -6326,7 +6326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:26">
+    <row r="80" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -6398,7 +6398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:26">
+    <row r="81" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -6470,7 +6470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:26">
+    <row r="82" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:26">
+    <row r="83" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -6614,7 +6614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:26">
+    <row r="84" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -6685,7 +6685,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="85" spans="1:26">
+    <row r="85" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -6757,7 +6757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:26">
+    <row r="86" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -6832,7 +6832,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="87" spans="1:26">
+    <row r="87" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -6904,7 +6904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:26">
+    <row r="88" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -6978,7 +6978,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="89" spans="1:26">
+    <row r="89" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -7050,7 +7050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:26">
+    <row r="90" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -7122,7 +7122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:26">
+    <row r="91" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
@@ -7194,7 +7194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:26">
+    <row r="92" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -7266,7 +7266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:26">
+    <row r="93" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -7338,7 +7338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:26">
+    <row r="94" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -7412,7 +7412,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="95" spans="1:26">
+    <row r="95" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -7484,7 +7484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:26">
+    <row r="96" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -7556,7 +7556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:23">
+    <row r="97" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
@@ -7627,7 +7627,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="98" spans="1:23">
+    <row r="98" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
@@ -7699,7 +7699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:23">
+    <row r="99" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
@@ -7771,7 +7771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:23">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
@@ -7843,7 +7843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:23">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
@@ -7915,7 +7915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:23">
+    <row r="102" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>101</v>
       </c>
@@ -7986,7 +7986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:23">
+    <row r="103" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>102</v>
       </c>
@@ -8058,7 +8058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:23">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>103</v>
       </c>
@@ -8130,7 +8130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:23">
+    <row r="105" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>104</v>
       </c>
@@ -8202,7 +8202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:23">
+    <row r="106" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>105</v>
       </c>
@@ -8274,7 +8274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:23">
+    <row r="107" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>106</v>
       </c>
@@ -8345,7 +8345,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" spans="1:23">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>107</v>
       </c>
@@ -8417,7 +8417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:23">
+    <row r="109" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
@@ -8489,7 +8489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:23">
+    <row r="110" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
@@ -8561,7 +8561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:23">
+    <row r="111" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
@@ -8633,7 +8633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:23">
+    <row r="112" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
@@ -8705,7 +8705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:26">
+    <row r="113" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
@@ -8780,7 +8780,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="114" spans="1:26">
+    <row r="114" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="115" spans="1:26">
+    <row r="115" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
@@ -8925,7 +8925,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="116" spans="1:26">
+    <row r="116" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
@@ -8999,7 +8999,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="117" spans="1:26">
+    <row r="117" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
@@ -9071,7 +9071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:26">
+    <row r="118" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
@@ -9143,7 +9143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:26">
+    <row r="119" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
@@ -9215,7 +9215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:26">
+    <row r="120" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>119</v>
       </c>
@@ -9287,7 +9287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:26">
+    <row r="121" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>120</v>
       </c>
@@ -9359,7 +9359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:26">
+    <row r="122" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>121</v>
       </c>
@@ -9434,7 +9434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:26">
+    <row r="123" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>122</v>
       </c>
@@ -9506,7 +9506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:26">
+    <row r="124" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>123</v>
       </c>
@@ -9578,7 +9578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:26">
+    <row r="125" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>124</v>
       </c>
@@ -9653,7 +9653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:26">
+    <row r="126" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>125</v>
       </c>
@@ -9728,7 +9728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:26">
+    <row r="127" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>126</v>
       </c>
@@ -9802,7 +9802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:26">
+    <row r="128" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>127</v>
       </c>
@@ -9876,7 +9876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:25">
+    <row r="129" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>128</v>
       </c>
@@ -9951,7 +9951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:25">
+    <row r="130" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>129</v>
       </c>
@@ -10023,7 +10023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:25">
+    <row r="131" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>130</v>
       </c>
@@ -10094,7 +10094,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132" spans="1:25">
+    <row r="132" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>131</v>
       </c>
@@ -10165,7 +10165,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="133" spans="1:25">
+    <row r="133" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>132</v>
       </c>
@@ -10236,7 +10236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:25">
+    <row r="134" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>133</v>
       </c>
@@ -10307,7 +10307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:25">
+    <row r="135" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>134</v>
       </c>
@@ -10378,7 +10378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:25">
+    <row r="136" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>135</v>
       </c>
@@ -10449,7 +10449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:25">
+    <row r="137" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>136</v>
       </c>
@@ -10520,7 +10520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:25">
+    <row r="138" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>137</v>
       </c>
@@ -10591,7 +10591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:25">
+    <row r="139" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>138</v>
       </c>
@@ -10662,7 +10662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:25">
+    <row r="140" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>139</v>
       </c>
@@ -10733,7 +10733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:25">
+    <row r="141" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>140</v>
       </c>
@@ -10804,7 +10804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:25">
+    <row r="142" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>141</v>
       </c>
@@ -10875,7 +10875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:25">
+    <row r="143" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>142</v>
       </c>
@@ -10946,7 +10946,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="144" spans="1:25">
+    <row r="144" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>143</v>
       </c>
@@ -11017,7 +11017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:26">
+    <row r="145" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>144</v>
       </c>
@@ -11088,7 +11088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:26">
+    <row r="146" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>145</v>
       </c>
@@ -11159,7 +11159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:26">
+    <row r="147" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>146</v>
       </c>
@@ -11230,7 +11230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:26">
+    <row r="148" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>147</v>
       </c>
@@ -11301,7 +11301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:26">
+    <row r="149" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>148</v>
       </c>
@@ -11372,7 +11372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:26">
+    <row r="150" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>149</v>
       </c>
@@ -11443,7 +11443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:26">
+    <row r="151" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>150</v>
       </c>
@@ -11514,7 +11514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:26">
+    <row r="152" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>151</v>
       </c>
@@ -11585,7 +11585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:26">
+    <row r="153" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>152</v>
       </c>
@@ -11656,7 +11656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:26">
+    <row r="154" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>153</v>
       </c>
@@ -11727,7 +11727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:26">
+    <row r="155" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>154</v>
       </c>
@@ -11798,7 +11798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:26">
+    <row r="156" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>155</v>
       </c>
@@ -11872,7 +11872,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="157" spans="1:26">
+    <row r="157" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>156</v>
       </c>
@@ -11943,7 +11943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:26">
+    <row r="158" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>157</v>
       </c>
@@ -12014,7 +12014,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="159" spans="1:26">
+    <row r="159" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>158</v>
       </c>
@@ -12085,7 +12085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:26">
+    <row r="160" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>159</v>
       </c>
@@ -12156,7 +12156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:23">
+    <row r="161" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>160</v>
       </c>
@@ -12227,7 +12227,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="162" spans="1:23">
+    <row r="162" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>161</v>
       </c>
@@ -12298,7 +12298,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="163" spans="1:23">
+    <row r="163" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>162</v>
       </c>
@@ -12369,7 +12369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="164" spans="1:23" s="3" customFormat="1">
+    <row r="164" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A164" s="3">
         <v>163</v>
       </c>
@@ -12440,7 +12440,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="165" spans="1:23">
+    <row r="165" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>164</v>
       </c>
@@ -12512,7 +12512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:23">
+    <row r="166" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>165</v>
       </c>
@@ -12584,7 +12584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:23">
+    <row r="167" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>166</v>
       </c>
@@ -12656,7 +12656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:23">
+    <row r="168" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>167</v>
       </c>
@@ -12728,7 +12728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:23">
+    <row r="169" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>168</v>
       </c>
@@ -12800,7 +12800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:23">
+    <row r="170" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>169</v>
       </c>
@@ -12872,7 +12872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:23">
+    <row r="171" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>170</v>
       </c>
@@ -12944,7 +12944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:23">
+    <row r="172" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>171</v>
       </c>
@@ -13015,7 +13015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:23">
+    <row r="173" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>172</v>
       </c>
@@ -13087,7 +13087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:23">
+    <row r="174" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>173</v>
       </c>
@@ -13158,7 +13158,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="175" spans="1:23">
+    <row r="175" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>174</v>
       </c>
@@ -13229,7 +13229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:23">
+    <row r="176" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>175</v>
       </c>
@@ -13301,7 +13301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:23">
+    <row r="177" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>176</v>
       </c>
@@ -13373,7 +13373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:23">
+    <row r="178" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>177</v>
       </c>
@@ -13444,7 +13444,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="179" spans="1:23">
+    <row r="179" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A179">
         <v>178</v>
       </c>
@@ -13515,7 +13515,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="180" spans="1:23">
+    <row r="180" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>179</v>
       </c>
@@ -13586,7 +13586,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="181" spans="1:23">
+    <row r="181" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>180</v>
       </c>
@@ -13658,7 +13658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:23">
+    <row r="182" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>181</v>
       </c>
@@ -13730,7 +13730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:23">
+    <row r="183" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A183">
         <v>182</v>
       </c>
@@ -13802,7 +13802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:23">
+    <row r="184" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>183</v>
       </c>
@@ -13873,7 +13873,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="185" spans="1:23">
+    <row r="185" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>184</v>
       </c>
@@ -13945,7 +13945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:23">
+    <row r="186" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>185</v>
       </c>
@@ -14017,7 +14017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:23">
+    <row r="187" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>186</v>
       </c>
@@ -14089,7 +14089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:23">
+    <row r="188" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>187</v>
       </c>
@@ -14161,7 +14161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:23">
+    <row r="189" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>188</v>
       </c>
@@ -14233,7 +14233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:23">
+    <row r="190" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>189</v>
       </c>
@@ -14305,7 +14305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:23">
+    <row r="191" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>190</v>
       </c>
@@ -14377,7 +14377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:23">
+    <row r="192" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>191</v>
       </c>
@@ -14448,7 +14448,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="193" spans="1:23">
+    <row r="193" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>192</v>
       </c>
@@ -14519,7 +14519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:23">
+    <row r="194" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>193</v>
       </c>
@@ -14590,7 +14590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:23">
+    <row r="195" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>194</v>
       </c>
@@ -14661,78 +14661,78 @@
         <v>28</v>
       </c>
     </row>
-    <row r="196" spans="1:23">
-      <c r="A196">
+    <row r="196" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A196" s="3">
         <v>195</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B196" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C196" t="s">
+      <c r="C196" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="4">
         <v>46076</v>
       </c>
-      <c r="E196" s="2">
+      <c r="E196" s="5">
         <v>0.47083333333333333</v>
       </c>
-      <c r="F196">
+      <c r="F196" s="3">
         <v>14.978</v>
       </c>
-      <c r="G196">
+      <c r="G196" s="3">
         <v>111.6</v>
       </c>
-      <c r="H196">
+      <c r="H196" s="3">
         <v>11.24</v>
       </c>
-      <c r="I196">
+      <c r="I196" s="3">
         <v>556</v>
       </c>
-      <c r="J196">
+      <c r="J196" s="3">
         <v>366.351</v>
       </c>
-      <c r="K196">
+      <c r="K196" s="3">
         <v>0.27</v>
       </c>
-      <c r="L196">
+      <c r="L196" s="3">
         <v>8.15</v>
       </c>
-      <c r="M196">
+      <c r="M196" s="3">
         <v>14.79</v>
       </c>
-      <c r="N196">
+      <c r="N196" s="3">
         <v>0.6</v>
       </c>
-      <c r="O196">
+      <c r="O196" s="3">
         <v>17.420000000000002</v>
       </c>
-      <c r="P196">
+      <c r="P196" s="3">
         <v>62.25</v>
       </c>
-      <c r="Q196" t="s">
-        <v>28</v>
-      </c>
-      <c r="R196" t="s">
-        <v>28</v>
-      </c>
-      <c r="S196" t="s">
-        <v>28</v>
-      </c>
-      <c r="T196" t="s">
-        <v>28</v>
-      </c>
-      <c r="U196" t="s">
-        <v>28</v>
-      </c>
-      <c r="V196" t="s">
-        <v>28</v>
-      </c>
-      <c r="W196" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="197" spans="1:23">
+      <c r="Q196" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R196" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="S196" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="T196" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="U196" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="V196" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="W196" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="197" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>196</v>
       </c>
@@ -14804,7 +14804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:23">
+    <row r="198" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>197</v>
       </c>
@@ -14876,7 +14876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:23">
+    <row r="199" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>198</v>
       </c>
@@ -14948,7 +14948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:23">
+    <row r="200" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>199</v>
       </c>
@@ -15020,7 +15020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="1:23">
+    <row r="201" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>200</v>
       </c>
@@ -15092,7 +15092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:23">
+    <row r="202" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>201</v>
       </c>
@@ -15164,7 +15164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:23">
+    <row r="203" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>202</v>
       </c>
@@ -15236,7 +15236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:23">
+    <row r="204" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A204">
         <v>203</v>
       </c>
@@ -15308,7 +15308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:23">
+    <row r="205" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A205">
         <v>204</v>
       </c>
@@ -15380,7 +15380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:23">
+    <row r="206" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A206">
         <v>205</v>
       </c>
@@ -15452,7 +15452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:23" ht="15">
+    <row r="207" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A207">
         <v>206</v>
       </c>
@@ -15523,7 +15523,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="208" spans="1:23">
+    <row r="208" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A208">
         <v>207</v>
       </c>
@@ -15594,7 +15594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:23">
+    <row r="209" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A209">
         <v>208</v>
       </c>
@@ -15665,7 +15665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:23">
+    <row r="210" spans="1:23" x14ac:dyDescent="0.35">
       <c r="D210" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed TEW sitetype error in point_wq.xlsx
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_point_wq.xlsx
+++ b/Data/tabular/YBLTE_point_wq.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Box\Yolo_Food_Web\Data\tabular\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Documents\R\Projects\YBLTE\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2416E154-FDFB-4B9B-878A-86C1F8869F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766FA540-7C25-4A10-B0EB-1D3A0FFF5659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="75">
   <si>
     <t>RowID</t>
   </si>
@@ -599,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z210"/>
+  <dimension ref="A1:Z222"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="12.453125" customWidth="1"/>
@@ -12090,7 +12090,7 @@
         <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="C160" t="s">
         <v>39</v>
@@ -15666,7 +15666,927 @@
       </c>
     </row>
     <row r="210" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="D210" s="1"/>
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" t="s">
+        <v>31</v>
+      </c>
+      <c r="C210" t="s">
+        <v>58</v>
+      </c>
+      <c r="D210" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E210" s="2">
+        <v>0.34513888888888888</v>
+      </c>
+      <c r="F210">
+        <v>15.343999999999999</v>
+      </c>
+      <c r="G210">
+        <v>100.4</v>
+      </c>
+      <c r="H210">
+        <v>10.039999999999999</v>
+      </c>
+      <c r="I210">
+        <v>470.3</v>
+      </c>
+      <c r="J210">
+        <v>305.72199999999998</v>
+      </c>
+      <c r="K210">
+        <v>0.23</v>
+      </c>
+      <c r="L210">
+        <v>8.5399999999999991</v>
+      </c>
+      <c r="M210">
+        <v>14.49</v>
+      </c>
+      <c r="N210">
+        <v>0.75</v>
+      </c>
+      <c r="O210">
+        <v>37.5</v>
+      </c>
+      <c r="P210">
+        <v>31.86</v>
+      </c>
+      <c r="Q210">
+        <v>3.5</v>
+      </c>
+      <c r="R210">
+        <v>30</v>
+      </c>
+      <c r="S210">
+        <v>4</v>
+      </c>
+      <c r="T210">
+        <v>23902</v>
+      </c>
+      <c r="U210">
+        <v>24435</v>
+      </c>
+      <c r="V210">
+        <v>533</v>
+      </c>
+      <c r="W210">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" t="s">
+        <v>31</v>
+      </c>
+      <c r="C211" t="s">
+        <v>32</v>
+      </c>
+      <c r="D211" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E211" s="2">
+        <v>0.37638888888888888</v>
+      </c>
+      <c r="F211">
+        <v>13.526999999999999</v>
+      </c>
+      <c r="G211">
+        <v>90.1</v>
+      </c>
+      <c r="H211">
+        <v>9.3699999999999992</v>
+      </c>
+      <c r="I211">
+        <v>165.7</v>
+      </c>
+      <c r="J211">
+        <v>107.726</v>
+      </c>
+      <c r="K211">
+        <v>0.08</v>
+      </c>
+      <c r="L211">
+        <v>7.65</v>
+      </c>
+      <c r="M211">
+        <v>63.61</v>
+      </c>
+      <c r="N211">
+        <v>0.17</v>
+      </c>
+      <c r="O211">
+        <v>0.93</v>
+      </c>
+      <c r="P211">
+        <v>20.5</v>
+      </c>
+      <c r="Q211">
+        <v>1.5</v>
+      </c>
+      <c r="R211">
+        <v>30</v>
+      </c>
+      <c r="S211">
+        <v>4</v>
+      </c>
+      <c r="T211">
+        <v>24435</v>
+      </c>
+      <c r="U211">
+        <v>25126</v>
+      </c>
+      <c r="V211">
+        <v>691</v>
+      </c>
+      <c r="W211">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" t="s">
+        <v>31</v>
+      </c>
+      <c r="C212" t="s">
+        <v>34</v>
+      </c>
+      <c r="D212" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E212" s="2">
+        <v>0.39374999999999999</v>
+      </c>
+      <c r="F212">
+        <v>13.683999999999999</v>
+      </c>
+      <c r="G212">
+        <v>94.2</v>
+      </c>
+      <c r="H212">
+        <v>9.77</v>
+      </c>
+      <c r="I212">
+        <v>168.8</v>
+      </c>
+      <c r="J212">
+        <v>109.714</v>
+      </c>
+      <c r="K212">
+        <v>0.08</v>
+      </c>
+      <c r="L212">
+        <v>7.72</v>
+      </c>
+      <c r="M212">
+        <v>64.209999999999994</v>
+      </c>
+      <c r="N212">
+        <v>0.19</v>
+      </c>
+      <c r="O212">
+        <v>0.84</v>
+      </c>
+      <c r="P212">
+        <v>20.010000000000002</v>
+      </c>
+      <c r="Q212">
+        <v>1.5</v>
+      </c>
+      <c r="R212">
+        <v>30</v>
+      </c>
+      <c r="S212">
+        <v>4</v>
+      </c>
+      <c r="T212">
+        <v>25132</v>
+      </c>
+      <c r="U212">
+        <v>25739</v>
+      </c>
+      <c r="V212">
+        <v>607</v>
+      </c>
+      <c r="W212">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" t="s">
+        <v>31</v>
+      </c>
+      <c r="C213" t="s">
+        <v>35</v>
+      </c>
+      <c r="D213" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E213" s="2">
+        <v>0.41458333333333336</v>
+      </c>
+      <c r="F213">
+        <v>14.507</v>
+      </c>
+      <c r="G213">
+        <v>82.1</v>
+      </c>
+      <c r="H213">
+        <v>8.36</v>
+      </c>
+      <c r="I213">
+        <v>318.89999999999998</v>
+      </c>
+      <c r="J213">
+        <v>207.29900000000001</v>
+      </c>
+      <c r="K213">
+        <v>0.15</v>
+      </c>
+      <c r="L213">
+        <v>7.7</v>
+      </c>
+      <c r="M213">
+        <v>46.93</v>
+      </c>
+      <c r="N213">
+        <v>0.21</v>
+      </c>
+      <c r="O213">
+        <v>4.58</v>
+      </c>
+      <c r="P213">
+        <v>42.54</v>
+      </c>
+      <c r="Q213">
+        <v>3.5</v>
+      </c>
+      <c r="R213">
+        <v>30</v>
+      </c>
+      <c r="S213">
+        <v>4</v>
+      </c>
+      <c r="T213">
+        <v>25739</v>
+      </c>
+      <c r="U213">
+        <v>26280</v>
+      </c>
+      <c r="V213">
+        <v>541</v>
+      </c>
+      <c r="W213">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" t="s">
+        <v>31</v>
+      </c>
+      <c r="C214" t="s">
+        <v>51</v>
+      </c>
+      <c r="D214" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E214" s="2">
+        <v>0.43541666666666667</v>
+      </c>
+      <c r="F214">
+        <v>15.423999999999999</v>
+      </c>
+      <c r="G214">
+        <v>91.9</v>
+      </c>
+      <c r="H214">
+        <v>9.18</v>
+      </c>
+      <c r="I214">
+        <v>273.60000000000002</v>
+      </c>
+      <c r="J214">
+        <v>177.83500000000001</v>
+      </c>
+      <c r="K214">
+        <v>0.13</v>
+      </c>
+      <c r="L214">
+        <v>7.83</v>
+      </c>
+      <c r="M214">
+        <v>53.78</v>
+      </c>
+      <c r="N214">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="O214">
+        <v>5.45</v>
+      </c>
+      <c r="P214">
+        <v>36.270000000000003</v>
+      </c>
+      <c r="Q214">
+        <v>3.5</v>
+      </c>
+      <c r="R214">
+        <v>30</v>
+      </c>
+      <c r="S214">
+        <v>4</v>
+      </c>
+      <c r="T214">
+        <v>26280</v>
+      </c>
+      <c r="U214">
+        <v>26819</v>
+      </c>
+      <c r="V214">
+        <v>539</v>
+      </c>
+      <c r="W214">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" t="s">
+        <v>31</v>
+      </c>
+      <c r="C215" t="s">
+        <v>53</v>
+      </c>
+      <c r="D215" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E215" s="2">
+        <v>0.44861111111111113</v>
+      </c>
+      <c r="F215">
+        <v>17.457999999999998</v>
+      </c>
+      <c r="G215">
+        <v>91.6</v>
+      </c>
+      <c r="H215">
+        <v>8.76</v>
+      </c>
+      <c r="I215">
+        <v>439.6</v>
+      </c>
+      <c r="J215">
+        <v>285.74299999999999</v>
+      </c>
+      <c r="K215">
+        <v>0.21</v>
+      </c>
+      <c r="L215">
+        <v>8.02</v>
+      </c>
+      <c r="M215">
+        <v>21.28</v>
+      </c>
+      <c r="N215">
+        <v>0.37</v>
+      </c>
+      <c r="O215">
+        <v>11.95</v>
+      </c>
+      <c r="P215">
+        <v>50.86</v>
+      </c>
+      <c r="Q215">
+        <v>5</v>
+      </c>
+      <c r="R215">
+        <v>30</v>
+      </c>
+      <c r="S215">
+        <v>4</v>
+      </c>
+      <c r="T215">
+        <v>26819</v>
+      </c>
+      <c r="U215">
+        <v>27447</v>
+      </c>
+      <c r="V215">
+        <v>628</v>
+      </c>
+      <c r="W215">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" t="s">
+        <v>31</v>
+      </c>
+      <c r="C216" t="s">
+        <v>36</v>
+      </c>
+      <c r="D216" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E216" s="2">
+        <v>0.48125000000000001</v>
+      </c>
+      <c r="F216">
+        <v>15.848000000000001</v>
+      </c>
+      <c r="G216">
+        <v>83.8</v>
+      </c>
+      <c r="H216">
+        <v>8.2899999999999991</v>
+      </c>
+      <c r="I216">
+        <v>231.2</v>
+      </c>
+      <c r="J216">
+        <v>150.202</v>
+      </c>
+      <c r="K216">
+        <v>0.11</v>
+      </c>
+      <c r="L216">
+        <v>7.63</v>
+      </c>
+      <c r="M216">
+        <v>55.28</v>
+      </c>
+      <c r="N216">
+        <v>0.27</v>
+      </c>
+      <c r="O216">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="P216">
+        <v>34.04</v>
+      </c>
+      <c r="Q216">
+        <v>3</v>
+      </c>
+      <c r="R216">
+        <v>30</v>
+      </c>
+      <c r="S216">
+        <v>4</v>
+      </c>
+      <c r="T216">
+        <v>27452</v>
+      </c>
+      <c r="U216">
+        <v>27972</v>
+      </c>
+      <c r="V216">
+        <v>520</v>
+      </c>
+      <c r="W216">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="s">
+        <v>31</v>
+      </c>
+      <c r="C217" t="s">
+        <v>38</v>
+      </c>
+      <c r="D217" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E217" s="2">
+        <v>0.51944444444444449</v>
+      </c>
+      <c r="F217">
+        <v>16.094999999999999</v>
+      </c>
+      <c r="G217">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="H217">
+        <v>6.93</v>
+      </c>
+      <c r="I217">
+        <v>195.5</v>
+      </c>
+      <c r="J217">
+        <v>127.04600000000001</v>
+      </c>
+      <c r="K217">
+        <v>0.09</v>
+      </c>
+      <c r="L217">
+        <v>7.4</v>
+      </c>
+      <c r="M217">
+        <v>56.13</v>
+      </c>
+      <c r="N217">
+        <v>0.33</v>
+      </c>
+      <c r="O217">
+        <v>9.08</v>
+      </c>
+      <c r="P217">
+        <v>38.6</v>
+      </c>
+      <c r="Q217">
+        <v>4</v>
+      </c>
+      <c r="R217">
+        <v>30</v>
+      </c>
+      <c r="S217">
+        <v>4</v>
+      </c>
+      <c r="T217">
+        <v>27982</v>
+      </c>
+      <c r="U217">
+        <v>28559</v>
+      </c>
+      <c r="V217">
+        <v>577</v>
+      </c>
+      <c r="W217">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" t="s">
+        <v>31</v>
+      </c>
+      <c r="C218" t="s">
+        <v>37</v>
+      </c>
+      <c r="D218" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E218" s="2">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F218">
+        <v>15.819000000000001</v>
+      </c>
+      <c r="G218">
+        <v>80.2</v>
+      </c>
+      <c r="H218">
+        <v>7.94</v>
+      </c>
+      <c r="I218">
+        <v>196.9</v>
+      </c>
+      <c r="J218">
+        <v>127.965</v>
+      </c>
+      <c r="K218">
+        <v>0.09</v>
+      </c>
+      <c r="L218">
+        <v>7.55</v>
+      </c>
+      <c r="M218">
+        <v>62.47</v>
+      </c>
+      <c r="N218">
+        <v>0.4</v>
+      </c>
+      <c r="O218">
+        <v>3.54</v>
+      </c>
+      <c r="P218">
+        <v>32.42</v>
+      </c>
+      <c r="Q218">
+        <v>3</v>
+      </c>
+      <c r="R218">
+        <v>30</v>
+      </c>
+      <c r="S218">
+        <v>4</v>
+      </c>
+      <c r="T218">
+        <v>28559</v>
+      </c>
+      <c r="U218">
+        <v>29242</v>
+      </c>
+      <c r="V218">
+        <v>683</v>
+      </c>
+      <c r="W218">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" t="s">
+        <v>31</v>
+      </c>
+      <c r="C219" t="s">
+        <v>46</v>
+      </c>
+      <c r="D219" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E219" s="2">
+        <v>0.375</v>
+      </c>
+      <c r="F219">
+        <v>17.224</v>
+      </c>
+      <c r="G219">
+        <v>63.2</v>
+      </c>
+      <c r="H219">
+        <v>6.07</v>
+      </c>
+      <c r="I219">
+        <v>610</v>
+      </c>
+      <c r="J219">
+        <v>396.488</v>
+      </c>
+      <c r="K219">
+        <v>0.3</v>
+      </c>
+      <c r="L219">
+        <v>7.72</v>
+      </c>
+      <c r="M219">
+        <v>17.25</v>
+      </c>
+      <c r="N219">
+        <v>0.48</v>
+      </c>
+      <c r="O219">
+        <v>8.7200000000000006</v>
+      </c>
+      <c r="P219">
+        <v>87.32</v>
+      </c>
+      <c r="Q219">
+        <v>2.5</v>
+      </c>
+      <c r="R219">
+        <v>30</v>
+      </c>
+      <c r="S219">
+        <v>4</v>
+      </c>
+      <c r="T219">
+        <v>18720</v>
+      </c>
+      <c r="U219">
+        <v>19301</v>
+      </c>
+      <c r="V219">
+        <v>581</v>
+      </c>
+      <c r="W219">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" t="s">
+        <v>31</v>
+      </c>
+      <c r="C220" t="s">
+        <v>48</v>
+      </c>
+      <c r="D220" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E220" s="2">
+        <v>0.40069444444444446</v>
+      </c>
+      <c r="F220">
+        <v>17.338999999999999</v>
+      </c>
+      <c r="G220">
+        <v>71.5</v>
+      </c>
+      <c r="H220">
+        <v>6.85</v>
+      </c>
+      <c r="I220">
+        <v>604</v>
+      </c>
+      <c r="J220">
+        <v>392.87700000000001</v>
+      </c>
+      <c r="K220">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="L220">
+        <v>7.75</v>
+      </c>
+      <c r="M220">
+        <v>16.27</v>
+      </c>
+      <c r="N220">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="O220">
+        <v>10.1</v>
+      </c>
+      <c r="P220">
+        <v>88.94</v>
+      </c>
+      <c r="Q220" t="s">
+        <v>28</v>
+      </c>
+      <c r="R220" t="s">
+        <v>28</v>
+      </c>
+      <c r="S220" t="s">
+        <v>28</v>
+      </c>
+      <c r="T220" t="s">
+        <v>28</v>
+      </c>
+      <c r="U220" t="s">
+        <v>28</v>
+      </c>
+      <c r="V220" t="s">
+        <v>28</v>
+      </c>
+      <c r="W220" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="221" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221" t="s">
+        <v>31</v>
+      </c>
+      <c r="C221" t="s">
+        <v>68</v>
+      </c>
+      <c r="D221" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E221" s="2">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="F221">
+        <v>16.568999999999999</v>
+      </c>
+      <c r="G221">
+        <v>91.8</v>
+      </c>
+      <c r="H221">
+        <v>8.94</v>
+      </c>
+      <c r="I221">
+        <v>481.4</v>
+      </c>
+      <c r="J221">
+        <v>312.92200000000003</v>
+      </c>
+      <c r="K221">
+        <v>0.23</v>
+      </c>
+      <c r="L221">
+        <v>7.66</v>
+      </c>
+      <c r="M221">
+        <v>50.06</v>
+      </c>
+      <c r="N221">
+        <v>1.23</v>
+      </c>
+      <c r="O221">
+        <v>31.81</v>
+      </c>
+      <c r="P221">
+        <v>74.87</v>
+      </c>
+      <c r="Q221">
+        <v>5</v>
+      </c>
+      <c r="R221">
+        <v>15</v>
+      </c>
+      <c r="S221">
+        <v>4</v>
+      </c>
+      <c r="T221" t="s">
+        <v>28</v>
+      </c>
+      <c r="U221" t="s">
+        <v>28</v>
+      </c>
+      <c r="V221" t="s">
+        <v>28</v>
+      </c>
+      <c r="W221">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" t="s">
+        <v>31</v>
+      </c>
+      <c r="C222" t="s">
+        <v>39</v>
+      </c>
+      <c r="D222" s="1">
+        <v>46084</v>
+      </c>
+      <c r="E222" s="2">
+        <v>0.52222222222222225</v>
+      </c>
+      <c r="F222">
+        <v>16.492999999999999</v>
+      </c>
+      <c r="G222">
+        <v>69.5</v>
+      </c>
+      <c r="H222">
+        <v>6.78</v>
+      </c>
+      <c r="I222">
+        <v>198.5</v>
+      </c>
+      <c r="J222">
+        <v>129.00299999999999</v>
+      </c>
+      <c r="K222">
+        <v>0.09</v>
+      </c>
+      <c r="L222">
+        <v>7.36</v>
+      </c>
+      <c r="M222">
+        <v>46.61</v>
+      </c>
+      <c r="N222">
+        <v>0.51</v>
+      </c>
+      <c r="O222">
+        <v>6.81</v>
+      </c>
+      <c r="P222">
+        <v>39.81</v>
+      </c>
+      <c r="Q222">
+        <v>3.5</v>
+      </c>
+      <c r="R222">
+        <v>30</v>
+      </c>
+      <c r="S222">
+        <v>4</v>
+      </c>
+      <c r="T222">
+        <v>19311</v>
+      </c>
+      <c r="U222">
+        <v>19703</v>
+      </c>
+      <c r="V222">
+        <v>392</v>
+      </c>
+      <c r="W222">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates to water quality, quantity, and logger scripts + data
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_point_wq.xlsx
+++ b/Data/tabular/YBLTE_point_wq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Documents\R\Projects\YBLTE\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED490F51-98E7-4318-A759-26B47CE2FB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41BFF2EE-8AA1-4920-8D59-41A0A0ED5C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="81">
   <si>
     <t>RowID</t>
   </si>
@@ -270,6 +270,15 @@
   </si>
   <si>
     <t>Sampled in EW fish passage channel</t>
+  </si>
+  <si>
+    <t>wq</t>
+  </si>
+  <si>
+    <t>ARC1</t>
+  </si>
+  <si>
+    <t>Backflow observed from Knaggs property to the KLRC channel near wq collection point just west of Wallace Weir.</t>
   </si>
 </sst>
 </file>
@@ -608,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z246"/>
+  <dimension ref="A1:Z258"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="12.453125" customWidth="1"/>
@@ -17911,7 +17920,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="241" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A241">
         <v>240</v>
       </c>
@@ -17982,7 +17991,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="242" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A242">
         <v>241</v>
       </c>
@@ -18053,7 +18062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A243">
         <v>242</v>
       </c>
@@ -18124,7 +18133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A244">
         <v>243</v>
       </c>
@@ -18195,7 +18204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A245">
         <v>244</v>
       </c>
@@ -18266,7 +18275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A246">
         <v>245</v>
       </c>
@@ -18334,6 +18343,861 @@
         <v>28</v>
       </c>
       <c r="W246">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A247">
+        <v>246</v>
+      </c>
+      <c r="B247" t="s">
+        <v>31</v>
+      </c>
+      <c r="C247" t="s">
+        <v>32</v>
+      </c>
+      <c r="D247" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E247" s="2">
+        <v>0.31874999999999998</v>
+      </c>
+      <c r="F247">
+        <v>18.649999999999999</v>
+      </c>
+      <c r="G247">
+        <v>93.3</v>
+      </c>
+      <c r="H247">
+        <v>8.7100000000000009</v>
+      </c>
+      <c r="I247">
+        <v>273.60000000000002</v>
+      </c>
+      <c r="J247">
+        <v>177.86600000000001</v>
+      </c>
+      <c r="K247">
+        <v>0.13</v>
+      </c>
+      <c r="L247">
+        <v>7.73</v>
+      </c>
+      <c r="M247">
+        <v>11.8</v>
+      </c>
+      <c r="N247">
+        <v>0.23</v>
+      </c>
+      <c r="O247">
+        <v>10.81</v>
+      </c>
+      <c r="P247">
+        <v>15.85</v>
+      </c>
+      <c r="Q247">
+        <v>2.5</v>
+      </c>
+      <c r="R247">
+        <v>30</v>
+      </c>
+      <c r="S247">
+        <v>4</v>
+      </c>
+      <c r="T247">
+        <v>201281</v>
+      </c>
+      <c r="U247">
+        <v>201883</v>
+      </c>
+      <c r="V247">
+        <v>602</v>
+      </c>
+      <c r="W247">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A248">
+        <v>247</v>
+      </c>
+      <c r="B248" t="s">
+        <v>69</v>
+      </c>
+      <c r="C248" t="s">
+        <v>73</v>
+      </c>
+      <c r="D248" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E248" s="2">
+        <v>0.3347222222222222</v>
+      </c>
+      <c r="F248">
+        <v>21.085000000000001</v>
+      </c>
+      <c r="G248">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="H248">
+        <v>6.65</v>
+      </c>
+      <c r="I248">
+        <v>640</v>
+      </c>
+      <c r="J248">
+        <v>416.25</v>
+      </c>
+      <c r="K248">
+        <v>0.31</v>
+      </c>
+      <c r="L248">
+        <v>7.68</v>
+      </c>
+      <c r="M248">
+        <v>7.27</v>
+      </c>
+      <c r="N248">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O248">
+        <v>6.71</v>
+      </c>
+      <c r="P248">
+        <v>22.28</v>
+      </c>
+      <c r="Q248" t="s">
+        <v>28</v>
+      </c>
+      <c r="R248" t="s">
+        <v>28</v>
+      </c>
+      <c r="S248" t="s">
+        <v>28</v>
+      </c>
+      <c r="T248" t="s">
+        <v>28</v>
+      </c>
+      <c r="U248" t="s">
+        <v>28</v>
+      </c>
+      <c r="V248" t="s">
+        <v>28</v>
+      </c>
+      <c r="W248">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A249">
+        <v>248</v>
+      </c>
+      <c r="B249" t="s">
+        <v>31</v>
+      </c>
+      <c r="C249" t="s">
+        <v>34</v>
+      </c>
+      <c r="D249" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E249" s="2">
+        <v>0.35555555555555557</v>
+      </c>
+      <c r="F249">
+        <v>21.084</v>
+      </c>
+      <c r="G249">
+        <v>69.8</v>
+      </c>
+      <c r="H249">
+        <v>6.2</v>
+      </c>
+      <c r="I249">
+        <v>623</v>
+      </c>
+      <c r="J249">
+        <v>404.80399999999997</v>
+      </c>
+      <c r="K249">
+        <v>0.3</v>
+      </c>
+      <c r="L249">
+        <v>7.61</v>
+      </c>
+      <c r="M249">
+        <v>5.83</v>
+      </c>
+      <c r="N249">
+        <v>0.12</v>
+      </c>
+      <c r="O249">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="P249">
+        <v>25.32</v>
+      </c>
+      <c r="Q249">
+        <v>3.5</v>
+      </c>
+      <c r="R249">
+        <v>30</v>
+      </c>
+      <c r="S249">
+        <v>4</v>
+      </c>
+      <c r="T249">
+        <v>201877</v>
+      </c>
+      <c r="U249">
+        <v>202849</v>
+      </c>
+      <c r="V249">
+        <v>972</v>
+      </c>
+      <c r="W249">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A250">
+        <v>249</v>
+      </c>
+      <c r="B250" t="s">
+        <v>78</v>
+      </c>
+      <c r="C250" t="s">
+        <v>79</v>
+      </c>
+      <c r="D250" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E250" s="2">
+        <v>0.36944444444444446</v>
+      </c>
+      <c r="F250">
+        <v>19.725999999999999</v>
+      </c>
+      <c r="G250">
+        <v>53.1</v>
+      </c>
+      <c r="H250">
+        <v>4.84</v>
+      </c>
+      <c r="I250">
+        <v>638</v>
+      </c>
+      <c r="J250">
+        <v>414.68599999999998</v>
+      </c>
+      <c r="K250">
+        <v>0.31</v>
+      </c>
+      <c r="L250">
+        <v>7.37</v>
+      </c>
+      <c r="M250">
+        <v>21.82</v>
+      </c>
+      <c r="N250">
+        <v>0.23</v>
+      </c>
+      <c r="O250">
+        <v>11.51</v>
+      </c>
+      <c r="P250">
+        <v>55.25</v>
+      </c>
+      <c r="Q250" t="s">
+        <v>28</v>
+      </c>
+      <c r="R250" t="s">
+        <v>28</v>
+      </c>
+      <c r="S250" t="s">
+        <v>28</v>
+      </c>
+      <c r="T250" t="s">
+        <v>28</v>
+      </c>
+      <c r="U250" t="s">
+        <v>28</v>
+      </c>
+      <c r="V250" t="s">
+        <v>28</v>
+      </c>
+      <c r="W250">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A251">
+        <v>250</v>
+      </c>
+      <c r="B251" t="s">
+        <v>31</v>
+      </c>
+      <c r="C251" t="s">
+        <v>35</v>
+      </c>
+      <c r="D251" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E251" s="2">
+        <v>0.39791666666666664</v>
+      </c>
+      <c r="F251">
+        <v>20.033999999999999</v>
+      </c>
+      <c r="G251">
+        <v>84.7</v>
+      </c>
+      <c r="H251">
+        <v>7.68</v>
+      </c>
+      <c r="I251">
+        <v>914</v>
+      </c>
+      <c r="J251">
+        <v>593.85500000000002</v>
+      </c>
+      <c r="K251">
+        <v>0.45</v>
+      </c>
+      <c r="L251">
+        <v>7.97</v>
+      </c>
+      <c r="M251">
+        <v>19.91</v>
+      </c>
+      <c r="N251">
+        <v>0.25</v>
+      </c>
+      <c r="O251">
+        <v>9.3699999999999992</v>
+      </c>
+      <c r="P251">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="Q251">
+        <v>3</v>
+      </c>
+      <c r="R251">
+        <v>30</v>
+      </c>
+      <c r="S251">
+        <v>4</v>
+      </c>
+      <c r="T251">
+        <v>202492</v>
+      </c>
+      <c r="U251">
+        <v>203035</v>
+      </c>
+      <c r="V251">
+        <v>543</v>
+      </c>
+      <c r="W251">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A252">
+        <v>251</v>
+      </c>
+      <c r="B252" t="s">
+        <v>31</v>
+      </c>
+      <c r="C252" t="s">
+        <v>51</v>
+      </c>
+      <c r="D252" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E252" s="2">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="F252">
+        <v>20.88</v>
+      </c>
+      <c r="G252">
+        <v>90.2</v>
+      </c>
+      <c r="H252">
+        <v>8.0399999999999991</v>
+      </c>
+      <c r="I252">
+        <v>956</v>
+      </c>
+      <c r="J252">
+        <v>621.39099999999996</v>
+      </c>
+      <c r="K252">
+        <v>0.47</v>
+      </c>
+      <c r="L252">
+        <v>8.26</v>
+      </c>
+      <c r="M252">
+        <v>8.65</v>
+      </c>
+      <c r="N252">
+        <v>0.09</v>
+      </c>
+      <c r="O252">
+        <v>2.5299999999999998</v>
+      </c>
+      <c r="P252">
+        <v>36.130000000000003</v>
+      </c>
+      <c r="Q252">
+        <v>2.5</v>
+      </c>
+      <c r="R252">
+        <v>15</v>
+      </c>
+      <c r="S252">
+        <v>4</v>
+      </c>
+      <c r="T252" t="s">
+        <v>28</v>
+      </c>
+      <c r="U252" t="s">
+        <v>28</v>
+      </c>
+      <c r="V252" t="s">
+        <v>28</v>
+      </c>
+      <c r="W252">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="253" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A253">
+        <v>253</v>
+      </c>
+      <c r="B253" t="s">
+        <v>78</v>
+      </c>
+      <c r="C253" t="s">
+        <v>48</v>
+      </c>
+      <c r="D253" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E253" s="2">
+        <v>0.31458333333333333</v>
+      </c>
+      <c r="F253">
+        <v>19.936</v>
+      </c>
+      <c r="G253">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="H253">
+        <v>1.78</v>
+      </c>
+      <c r="I253">
+        <v>1795</v>
+      </c>
+      <c r="J253">
+        <v>1167.037</v>
+      </c>
+      <c r="K253">
+        <v>0.91</v>
+      </c>
+      <c r="L253">
+        <v>8</v>
+      </c>
+      <c r="M253">
+        <v>8.77</v>
+      </c>
+      <c r="N253">
+        <v>0.21</v>
+      </c>
+      <c r="O253">
+        <v>4.17</v>
+      </c>
+      <c r="P253">
+        <v>117.49</v>
+      </c>
+      <c r="Q253">
+        <v>4</v>
+      </c>
+      <c r="R253">
+        <v>30</v>
+      </c>
+      <c r="S253">
+        <v>4</v>
+      </c>
+      <c r="T253">
+        <v>48487</v>
+      </c>
+      <c r="U253">
+        <v>48958</v>
+      </c>
+      <c r="V253">
+        <v>471</v>
+      </c>
+      <c r="W253">
+        <v>1</v>
+      </c>
+      <c r="Z253" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="254" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A254">
+        <v>254</v>
+      </c>
+      <c r="B254" t="s">
+        <v>31</v>
+      </c>
+      <c r="C254" t="s">
+        <v>58</v>
+      </c>
+      <c r="D254" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E254" s="2">
+        <v>0.33888888888888891</v>
+      </c>
+      <c r="F254">
+        <v>19.341999999999999</v>
+      </c>
+      <c r="G254">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="H254">
+        <v>7.2</v>
+      </c>
+      <c r="I254">
+        <v>816</v>
+      </c>
+      <c r="J254">
+        <v>530.73699999999997</v>
+      </c>
+      <c r="K254">
+        <v>0.4</v>
+      </c>
+      <c r="L254">
+        <v>8.11</v>
+      </c>
+      <c r="M254">
+        <v>28.92</v>
+      </c>
+      <c r="N254">
+        <v>0.3</v>
+      </c>
+      <c r="O254">
+        <v>8.36</v>
+      </c>
+      <c r="P254">
+        <v>28.81</v>
+      </c>
+      <c r="Q254">
+        <v>4.5</v>
+      </c>
+      <c r="R254">
+        <v>30</v>
+      </c>
+      <c r="S254">
+        <v>4</v>
+      </c>
+      <c r="T254">
+        <v>48959</v>
+      </c>
+      <c r="U254">
+        <v>49549</v>
+      </c>
+      <c r="V254">
+        <v>590</v>
+      </c>
+      <c r="W254">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A255">
+        <v>255</v>
+      </c>
+      <c r="B255" t="s">
+        <v>31</v>
+      </c>
+      <c r="C255" t="s">
+        <v>38</v>
+      </c>
+      <c r="D255" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E255" s="2">
+        <v>0.38819444444444445</v>
+      </c>
+      <c r="F255">
+        <v>21.306000000000001</v>
+      </c>
+      <c r="G255">
+        <v>54.3</v>
+      </c>
+      <c r="H255">
+        <v>4.79</v>
+      </c>
+      <c r="I255">
+        <v>689</v>
+      </c>
+      <c r="J255">
+        <v>447.61399999999998</v>
+      </c>
+      <c r="K255">
+        <v>0.34</v>
+      </c>
+      <c r="L255">
+        <v>7.75</v>
+      </c>
+      <c r="M255">
+        <v>8.24</v>
+      </c>
+      <c r="N255">
+        <v>0.15</v>
+      </c>
+      <c r="O255">
+        <v>4.29</v>
+      </c>
+      <c r="P255">
+        <v>63.02</v>
+      </c>
+      <c r="Q255">
+        <v>3</v>
+      </c>
+      <c r="R255">
+        <v>30</v>
+      </c>
+      <c r="S255">
+        <v>4</v>
+      </c>
+      <c r="T255">
+        <v>49595</v>
+      </c>
+      <c r="U255">
+        <v>50085</v>
+      </c>
+      <c r="V255">
+        <v>490</v>
+      </c>
+      <c r="W255">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A256">
+        <v>256</v>
+      </c>
+      <c r="B256" t="s">
+        <v>31</v>
+      </c>
+      <c r="C256" t="s">
+        <v>39</v>
+      </c>
+      <c r="D256" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E256" s="2">
+        <v>0.42569444444444443</v>
+      </c>
+      <c r="F256">
+        <v>19.036000000000001</v>
+      </c>
+      <c r="G256">
+        <v>43.3</v>
+      </c>
+      <c r="H256">
+        <v>4</v>
+      </c>
+      <c r="I256">
+        <v>594</v>
+      </c>
+      <c r="J256">
+        <v>386</v>
+      </c>
+      <c r="K256">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="L256">
+        <v>7.55</v>
+      </c>
+      <c r="M256">
+        <v>6.98</v>
+      </c>
+      <c r="N256">
+        <v>0.31</v>
+      </c>
+      <c r="O256">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="P256">
+        <v>93.33</v>
+      </c>
+      <c r="Q256">
+        <v>5</v>
+      </c>
+      <c r="R256">
+        <v>15</v>
+      </c>
+      <c r="S256">
+        <v>4</v>
+      </c>
+      <c r="T256" t="s">
+        <v>28</v>
+      </c>
+      <c r="U256" t="s">
+        <v>28</v>
+      </c>
+      <c r="V256" t="s">
+        <v>28</v>
+      </c>
+      <c r="W256">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A257">
+        <v>257</v>
+      </c>
+      <c r="B257" t="s">
+        <v>31</v>
+      </c>
+      <c r="C257" t="s">
+        <v>37</v>
+      </c>
+      <c r="D257" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E257" s="2">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="F257">
+        <v>21.63</v>
+      </c>
+      <c r="G257">
+        <v>53.6</v>
+      </c>
+      <c r="H257">
+        <v>4.71</v>
+      </c>
+      <c r="I257">
+        <v>778</v>
+      </c>
+      <c r="J257">
+        <v>505.78500000000003</v>
+      </c>
+      <c r="K257">
+        <v>0.38</v>
+      </c>
+      <c r="L257">
+        <v>7.75</v>
+      </c>
+      <c r="M257">
+        <v>14.25</v>
+      </c>
+      <c r="N257">
+        <v>0.43</v>
+      </c>
+      <c r="O257">
+        <v>9.08</v>
+      </c>
+      <c r="P257">
+        <v>55.42</v>
+      </c>
+      <c r="Q257">
+        <v>3</v>
+      </c>
+      <c r="R257">
+        <v>30</v>
+      </c>
+      <c r="S257">
+        <v>4</v>
+      </c>
+      <c r="T257">
+        <v>51792</v>
+      </c>
+      <c r="U257">
+        <v>52457</v>
+      </c>
+      <c r="V257">
+        <v>665</v>
+      </c>
+      <c r="W257">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="258" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A258">
+        <v>258</v>
+      </c>
+      <c r="B258" t="s">
+        <v>31</v>
+      </c>
+      <c r="C258" t="s">
+        <v>36</v>
+      </c>
+      <c r="D258" s="1">
+        <v>46105</v>
+      </c>
+      <c r="E258" s="2">
+        <v>0.49513888888888891</v>
+      </c>
+      <c r="F258">
+        <v>22.888000000000002</v>
+      </c>
+      <c r="G258">
+        <v>53</v>
+      </c>
+      <c r="H258">
+        <v>4.54</v>
+      </c>
+      <c r="I258">
+        <v>860</v>
+      </c>
+      <c r="J258">
+        <v>559.26400000000001</v>
+      </c>
+      <c r="K258">
+        <v>0.42</v>
+      </c>
+      <c r="L258">
+        <v>7.79</v>
+      </c>
+      <c r="M258">
+        <v>16.59</v>
+      </c>
+      <c r="N258">
+        <v>0.2</v>
+      </c>
+      <c r="O258">
+        <v>4.47</v>
+      </c>
+      <c r="P258">
+        <v>51.61</v>
+      </c>
+      <c r="Q258">
+        <v>3</v>
+      </c>
+      <c r="R258">
+        <v>30</v>
+      </c>
+      <c r="S258">
+        <v>4</v>
+      </c>
+      <c r="T258">
+        <v>52458</v>
+      </c>
+      <c r="U258">
+        <v>53078</v>
+      </c>
+      <c r="V258">
+        <v>620</v>
+      </c>
+      <c r="W258">
         <v>1</v>
       </c>
     </row>

</xml_diff>